<commit_message>
criado novo arquivo .xlsx com mais 5000 novos dados de empresas.
</commit_message>
<xml_diff>
--- a/output_data_cnae/resultado_consulta_cnae_Ubuntu_erros.xlsx
+++ b/output_data_cnae/resultado_consulta_cnae_Ubuntu_erros.xlsx
@@ -56,7 +56,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -83,14 +83,6 @@
       <b val="true"/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <u val="single"/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -120,7 +112,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="21">
+  <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -144,11 +136,8 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -157,19 +146,14 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
 </styleSheet>
 </file>
@@ -354,7 +338,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -385,48 +369,6 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F3" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F4" s="2"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F5" s="2"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F6" s="2"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F7" s="2"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F8" s="2"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F9" s="2"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F10" s="2"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F12" s="2"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F13" s="2"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F14" s="2"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F15" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>